<commit_message>
NX5e HVAC RPM 작성 완료
</commit_message>
<xml_diff>
--- a/7. 모델별 RPM/HKMC_AIR_PTC_모델별_HVAC_RPM.xlsx
+++ b/7. 모델별 RPM/HKMC_AIR_PTC_모델별_HVAC_RPM.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\PROJECT\Gitlab\HMC\ptc_heater_doc\7. 모델별 RPM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\일정\ptc_heater_doc\7. 모델별 RPM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11760"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11760" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="이력관리" sheetId="8" r:id="rId1"/>
@@ -20,9 +20,9 @@
     <sheet name="KY" sheetId="6" r:id="rId6"/>
     <sheet name="Su2i" sheetId="10" r:id="rId7"/>
     <sheet name="QV" sheetId="5" r:id="rId8"/>
+    <sheet name="NX5e" sheetId="11" r:id="rId9"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
   </externalReferences>
   <definedNames>
@@ -31,27 +31,34 @@
     <definedName name="A">[1]hp_td_calc!$D$7:$W$7</definedName>
     <definedName name="B">[1]hp_td_calc!$D$8:$W$8</definedName>
     <definedName name="BLOWER" localSheetId="4">#REF!</definedName>
+    <definedName name="BLOWER" localSheetId="8">#REF!</definedName>
     <definedName name="BLOWER" localSheetId="6">#REF!</definedName>
     <definedName name="BLOWER">#REF!</definedName>
     <definedName name="D">[1]hp_td_calc!$D$10:$W$10</definedName>
     <definedName name="Fset">[1]hp_td_calc!$D$12:$W$12</definedName>
     <definedName name="fuseopen" localSheetId="4">#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!</definedName>
+    <definedName name="fuseopen" localSheetId="8">#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!</definedName>
     <definedName name="fuseopen" localSheetId="6">#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!</definedName>
     <definedName name="fuseopen">#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!,#REF!</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">이력관리!$A$1:$K$24</definedName>
     <definedName name="pull" localSheetId="4">#REF!</definedName>
+    <definedName name="pull" localSheetId="8">#REF!</definedName>
     <definedName name="pull" localSheetId="6">#REF!</definedName>
     <definedName name="pull">#REF!</definedName>
     <definedName name="pull_m10" localSheetId="4">#REF!</definedName>
+    <definedName name="pull_m10" localSheetId="8">#REF!</definedName>
     <definedName name="pull_m10" localSheetId="6">#REF!</definedName>
     <definedName name="pull_m10">#REF!</definedName>
     <definedName name="pull_m5" localSheetId="4">#REF!</definedName>
+    <definedName name="pull_m5" localSheetId="8">#REF!</definedName>
     <definedName name="pull_m5" localSheetId="6">#REF!</definedName>
     <definedName name="pull_m5">#REF!</definedName>
     <definedName name="pull_p10" localSheetId="4">#REF!</definedName>
+    <definedName name="pull_p10" localSheetId="8">#REF!</definedName>
     <definedName name="pull_p10" localSheetId="6">#REF!</definedName>
     <definedName name="pull_p10">#REF!</definedName>
     <definedName name="Puu_p5" localSheetId="4">#REF!</definedName>
+    <definedName name="Puu_p5" localSheetId="8">#REF!</definedName>
     <definedName name="Puu_p5" localSheetId="6">#REF!</definedName>
     <definedName name="Puu_p5">#REF!</definedName>
     <definedName name="Tamb">[1]hp_td_calc!$D$13:$W$13</definedName>
@@ -82,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="60">
   <si>
     <t>VENT</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -297,6 +304,26 @@
   </si>
   <si>
     <t>QV HVAC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NX5e HVAC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VENT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FLOOR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>25. 10. 21. FLOOR 모드 한온 이호 전임 답변</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>25. 10. 22. VENT 모드 한온 이호 전임 답변</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -307,8 +334,8 @@
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="0&quot;단&quot;"/>
     <numFmt numFmtId="177" formatCode="0&quot;RPM&quot;"/>
-    <numFmt numFmtId="182" formatCode="0.0&quot;V&quot;"/>
-    <numFmt numFmtId="184" formatCode="0&quot;%&quot;"/>
+    <numFmt numFmtId="178" formatCode="0.0&quot;V&quot;"/>
+    <numFmt numFmtId="179" formatCode="0&quot;%&quot;"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -381,7 +408,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="45">
+  <borders count="47">
     <border>
       <left/>
       <right/>
@@ -951,6 +978,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -959,16 +1006,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -984,54 +1028,30 @@
     <xf numFmtId="176" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
     <xf numFmtId="177" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="177" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -1041,42 +1061,18 @@
     <xf numFmtId="177" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1084,103 +1080,28 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="2" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="184" fontId="3" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="184" fontId="3" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="184" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="184" fontId="3" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="184" fontId="3" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="184" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="184" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="184" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="184" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="3" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="177" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
@@ -1191,25 +1112,10 @@
     <xf numFmtId="177" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="3" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1228,31 +1134,22 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="3" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="3" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="3" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="6" fillId="0" borderId="3" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1264,15 +1161,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
@@ -1282,31 +1170,202 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="3" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1340,37 +1399,6 @@
       <sheetData sheetId="0" refreshError="1"/>
       <sheetData sheetId="1" refreshError="1"/>
       <sheetData sheetId="2" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
-<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="표지"/>
-      <sheetName val="이력관리"/>
-      <sheetName val="목차"/>
-      <sheetName val="1.형상 및 커넥터"/>
-      <sheetName val="2.Block Diagram"/>
-      <sheetName val="3. 작동 Logic"/>
-      <sheetName val="4. FAIL SAFE"/>
-      <sheetName val="5.FLOWCHART"/>
-      <sheetName val="6.전원onoff시 PTC수행기능"/>
-      <sheetName val="7.Local CAN DB"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1645,268 +1673,291 @@
   <dimension ref="A1:I21"/>
   <sheetFormatPr defaultColWidth="2.375" defaultRowHeight="12" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.875" style="88" customWidth="1"/>
-    <col min="2" max="2" width="6.875" style="88" customWidth="1"/>
-    <col min="3" max="3" width="6.375" style="88" customWidth="1"/>
-    <col min="4" max="4" width="18.375" style="88" customWidth="1"/>
-    <col min="5" max="5" width="20" style="88" customWidth="1"/>
-    <col min="6" max="6" width="9.5" style="88" customWidth="1"/>
-    <col min="7" max="7" width="5.5" style="88" customWidth="1"/>
-    <col min="8" max="8" width="4" style="88" customWidth="1"/>
-    <col min="9" max="9" width="9.125" style="88" customWidth="1"/>
-    <col min="10" max="10" width="0.875" style="88" customWidth="1"/>
-    <col min="11" max="16384" width="2.375" style="88"/>
+    <col min="1" max="1" width="11.875" style="41" customWidth="1"/>
+    <col min="2" max="2" width="6.875" style="41" customWidth="1"/>
+    <col min="3" max="3" width="6.375" style="41" customWidth="1"/>
+    <col min="4" max="4" width="18.375" style="41" customWidth="1"/>
+    <col min="5" max="5" width="20" style="41" customWidth="1"/>
+    <col min="6" max="6" width="9.5" style="41" customWidth="1"/>
+    <col min="7" max="7" width="5.5" style="41" customWidth="1"/>
+    <col min="8" max="8" width="4" style="41" customWidth="1"/>
+    <col min="9" max="9" width="9.125" style="41" customWidth="1"/>
+    <col min="10" max="10" width="0.875" style="41" customWidth="1"/>
+    <col min="11" max="16384" width="2.375" style="41"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="87" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="1" spans="1:9" s="40" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="101" t="s">
+      <c r="A2" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="101"/>
-      <c r="C2" s="101"/>
-      <c r="D2" s="101"/>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="101"/>
-      <c r="H2" s="101"/>
-      <c r="I2" s="101"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
     </row>
     <row r="3" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="101" t="s">
+      <c r="A3" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="101"/>
-      <c r="C3" s="101"/>
-      <c r="D3" s="102" t="s">
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="102" t="s">
+      <c r="E3" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="101" t="s">
+      <c r="F3" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="101"/>
-      <c r="H3" s="101"/>
-      <c r="I3" s="101"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
     </row>
     <row r="4" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="92" t="s">
+      <c r="A4" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="93" t="s">
+      <c r="B4" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="89" t="s">
+      <c r="C4" s="54" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="91"/>
-      <c r="E4" s="90"/>
-      <c r="F4" s="94" t="s">
+      <c r="D4" s="55"/>
+      <c r="E4" s="56"/>
+      <c r="F4" s="57" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="103"/>
-      <c r="H4" s="103"/>
-      <c r="I4" s="95"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="59"/>
     </row>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="96" t="s">
+      <c r="A5" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="97" t="s">
+      <c r="B5" s="45" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="98" t="s">
+      <c r="C5" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="99"/>
-      <c r="E5" s="100"/>
-      <c r="F5" s="104" t="s">
+      <c r="D5" s="49"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="51" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="105"/>
-      <c r="H5" s="105"/>
-      <c r="I5" s="106"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+      <c r="I5" s="53"/>
     </row>
     <row r="6" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="96"/>
-      <c r="B6" s="97"/>
-      <c r="C6" s="98"/>
-      <c r="D6" s="99"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="104"/>
-      <c r="G6" s="105"/>
-      <c r="H6" s="105"/>
-      <c r="I6" s="106"/>
+      <c r="A6" s="44"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="48"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="51"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="53"/>
     </row>
     <row r="7" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="96"/>
-      <c r="B7" s="97"/>
-      <c r="C7" s="98"/>
-      <c r="D7" s="99"/>
-      <c r="E7" s="100"/>
-      <c r="F7" s="104"/>
-      <c r="G7" s="105"/>
-      <c r="H7" s="105"/>
-      <c r="I7" s="106"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="48"/>
+      <c r="D7" s="49"/>
+      <c r="E7" s="50"/>
+      <c r="F7" s="51"/>
+      <c r="G7" s="52"/>
+      <c r="H7" s="52"/>
+      <c r="I7" s="53"/>
     </row>
     <row r="8" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="96"/>
-      <c r="B8" s="97"/>
-      <c r="C8" s="98"/>
-      <c r="D8" s="99"/>
-      <c r="E8" s="100"/>
-      <c r="F8" s="104"/>
-      <c r="G8" s="105"/>
-      <c r="H8" s="105"/>
-      <c r="I8" s="106"/>
+      <c r="A8" s="44"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="48"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="51"/>
+      <c r="G8" s="52"/>
+      <c r="H8" s="52"/>
+      <c r="I8" s="53"/>
     </row>
     <row r="9" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="96"/>
-      <c r="B9" s="97"/>
-      <c r="C9" s="98"/>
-      <c r="D9" s="99"/>
-      <c r="E9" s="100"/>
-      <c r="F9" s="104"/>
-      <c r="G9" s="105"/>
-      <c r="H9" s="105"/>
-      <c r="I9" s="106"/>
+      <c r="A9" s="44"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="52"/>
+      <c r="H9" s="52"/>
+      <c r="I9" s="53"/>
     </row>
     <row r="10" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="96"/>
-      <c r="B10" s="97"/>
-      <c r="C10" s="98"/>
-      <c r="D10" s="99"/>
-      <c r="E10" s="100"/>
-      <c r="F10" s="104"/>
-      <c r="G10" s="105"/>
-      <c r="H10" s="105"/>
-      <c r="I10" s="106"/>
+      <c r="A10" s="44"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="50"/>
+      <c r="F10" s="51"/>
+      <c r="G10" s="52"/>
+      <c r="H10" s="52"/>
+      <c r="I10" s="53"/>
     </row>
     <row r="11" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="96"/>
-      <c r="B11" s="97"/>
-      <c r="C11" s="98"/>
-      <c r="D11" s="99"/>
-      <c r="E11" s="100"/>
-      <c r="F11" s="104"/>
-      <c r="G11" s="105"/>
-      <c r="H11" s="105"/>
-      <c r="I11" s="106"/>
+      <c r="A11" s="44"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="51"/>
+      <c r="G11" s="52"/>
+      <c r="H11" s="52"/>
+      <c r="I11" s="53"/>
     </row>
     <row r="12" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="96"/>
-      <c r="B12" s="97"/>
-      <c r="C12" s="98"/>
-      <c r="D12" s="99"/>
-      <c r="E12" s="100"/>
-      <c r="F12" s="104"/>
-      <c r="G12" s="105"/>
-      <c r="H12" s="105"/>
-      <c r="I12" s="106"/>
+      <c r="A12" s="44"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="51"/>
+      <c r="G12" s="52"/>
+      <c r="H12" s="52"/>
+      <c r="I12" s="53"/>
     </row>
     <row r="13" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="96"/>
-      <c r="B13" s="97"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="99"/>
-      <c r="E13" s="100"/>
-      <c r="F13" s="104"/>
-      <c r="G13" s="105"/>
-      <c r="H13" s="105"/>
-      <c r="I13" s="106"/>
+      <c r="A13" s="44"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="48"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="52"/>
+      <c r="H13" s="52"/>
+      <c r="I13" s="53"/>
     </row>
     <row r="14" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="96"/>
-      <c r="B14" s="97"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="99"/>
-      <c r="E14" s="100"/>
-      <c r="F14" s="104"/>
-      <c r="G14" s="105"/>
-      <c r="H14" s="105"/>
-      <c r="I14" s="106"/>
+      <c r="A14" s="44"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="52"/>
+      <c r="H14" s="52"/>
+      <c r="I14" s="53"/>
     </row>
     <row r="15" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="96"/>
-      <c r="B15" s="97"/>
-      <c r="C15" s="98"/>
-      <c r="D15" s="99"/>
-      <c r="E15" s="100"/>
-      <c r="F15" s="104"/>
-      <c r="G15" s="105"/>
-      <c r="H15" s="105"/>
-      <c r="I15" s="106"/>
+      <c r="A15" s="44"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="52"/>
+      <c r="I15" s="53"/>
     </row>
     <row r="16" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="96"/>
-      <c r="B16" s="97"/>
-      <c r="C16" s="98"/>
-      <c r="D16" s="99"/>
-      <c r="E16" s="100"/>
-      <c r="F16" s="104"/>
-      <c r="G16" s="105"/>
-      <c r="H16" s="105"/>
-      <c r="I16" s="106"/>
+      <c r="A16" s="44"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="51"/>
+      <c r="G16" s="52"/>
+      <c r="H16" s="52"/>
+      <c r="I16" s="53"/>
     </row>
     <row r="17" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="96"/>
-      <c r="B17" s="97"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="99"/>
-      <c r="E17" s="100"/>
-      <c r="F17" s="104"/>
-      <c r="G17" s="105"/>
-      <c r="H17" s="105"/>
-      <c r="I17" s="106"/>
+      <c r="A17" s="44"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="48"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="52"/>
+      <c r="H17" s="52"/>
+      <c r="I17" s="53"/>
     </row>
     <row r="18" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="96"/>
-      <c r="B18" s="97"/>
-      <c r="C18" s="98"/>
-      <c r="D18" s="99"/>
-      <c r="E18" s="100"/>
-      <c r="F18" s="104"/>
-      <c r="G18" s="105"/>
-      <c r="H18" s="105"/>
-      <c r="I18" s="106"/>
+      <c r="A18" s="44"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="48"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="52"/>
+      <c r="H18" s="52"/>
+      <c r="I18" s="53"/>
     </row>
     <row r="19" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="96"/>
-      <c r="B19" s="97"/>
-      <c r="C19" s="98"/>
-      <c r="D19" s="99"/>
-      <c r="E19" s="100"/>
-      <c r="F19" s="104"/>
-      <c r="G19" s="105"/>
-      <c r="H19" s="105"/>
-      <c r="I19" s="106"/>
+      <c r="A19" s="44"/>
+      <c r="B19" s="45"/>
+      <c r="C19" s="48"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="51"/>
+      <c r="G19" s="52"/>
+      <c r="H19" s="52"/>
+      <c r="I19" s="53"/>
     </row>
     <row r="20" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="96"/>
-      <c r="B20" s="97"/>
-      <c r="C20" s="98"/>
-      <c r="D20" s="99"/>
-      <c r="E20" s="100"/>
-      <c r="F20" s="104"/>
-      <c r="G20" s="105"/>
-      <c r="H20" s="105"/>
-      <c r="I20" s="106"/>
+      <c r="A20" s="44"/>
+      <c r="B20" s="45"/>
+      <c r="C20" s="48"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="51"/>
+      <c r="G20" s="52"/>
+      <c r="H20" s="52"/>
+      <c r="I20" s="53"/>
     </row>
     <row r="21" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="96"/>
-      <c r="B21" s="97"/>
-      <c r="C21" s="98"/>
-      <c r="D21" s="99"/>
-      <c r="E21" s="100"/>
-      <c r="F21" s="104"/>
-      <c r="G21" s="105"/>
-      <c r="H21" s="105"/>
-      <c r="I21" s="106"/>
+      <c r="A21" s="44"/>
+      <c r="B21" s="45"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
+      <c r="H21" s="52"/>
+      <c r="I21" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="F6:I6"/>
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="F5:I5"/>
+    <mergeCell ref="C8:E8"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="C10:E10"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="C11:E11"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F11:I11"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="F13:I13"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="F3:I3"/>
     <mergeCell ref="C20:E20"/>
@@ -1923,29 +1974,6 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F14:I14"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="C11:E11"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C13:E13"/>
-    <mergeCell ref="F11:I11"/>
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="C10:E10"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C7:E7"/>
-    <mergeCell ref="F6:I6"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="F5:I5"/>
-    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.74803149606299213" right="0.15748031496062992" top="0.78740157480314965" bottom="0.72" header="0.51181102362204722" footer="0.51181102362204722"/>
@@ -1968,359 +1996,355 @@
   <sheetData>
     <row r="4" spans="2:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="75" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="12"/>
+      <c r="C5" s="76"/>
+      <c r="D5" s="76"/>
+      <c r="E5" s="76"/>
+      <c r="F5" s="76"/>
+      <c r="G5" s="77"/>
     </row>
     <row r="6" spans="2:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B7" s="13">
+      <c r="B7" s="8">
         <v>1</v>
       </c>
-      <c r="C7" s="72">
+      <c r="C7" s="69">
         <v>1107</v>
       </c>
-      <c r="D7" s="73"/>
-      <c r="E7" s="72">
+      <c r="D7" s="70"/>
+      <c r="E7" s="69">
         <v>1457</v>
       </c>
-      <c r="F7" s="73"/>
-      <c r="G7" s="74">
+      <c r="F7" s="70"/>
+      <c r="G7" s="32">
         <v>1473</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="70">
+      <c r="C8" s="67">
         <v>1360</v>
       </c>
-      <c r="D8" s="71"/>
-      <c r="E8" s="70">
+      <c r="D8" s="68"/>
+      <c r="E8" s="67">
         <v>1610</v>
       </c>
-      <c r="F8" s="71"/>
-      <c r="G8" s="75">
+      <c r="F8" s="68"/>
+      <c r="G8" s="33">
         <v>1660</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B9" s="5">
+      <c r="B9" s="4">
         <v>3</v>
       </c>
-      <c r="C9" s="70">
+      <c r="C9" s="67">
         <v>1600</v>
       </c>
-      <c r="D9" s="71"/>
-      <c r="E9" s="70">
+      <c r="D9" s="68"/>
+      <c r="E9" s="67">
         <v>1740</v>
       </c>
-      <c r="F9" s="71"/>
-      <c r="G9" s="75">
+      <c r="F9" s="68"/>
+      <c r="G9" s="33">
         <v>1940</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B10" s="5">
+      <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="70">
+      <c r="C10" s="67">
         <v>1840</v>
       </c>
-      <c r="D10" s="71"/>
-      <c r="E10" s="70">
+      <c r="D10" s="68"/>
+      <c r="E10" s="67">
         <v>1960</v>
       </c>
-      <c r="F10" s="71"/>
-      <c r="G10" s="75">
+      <c r="F10" s="68"/>
+      <c r="G10" s="33">
         <v>2120</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>5</v>
       </c>
-      <c r="C11" s="70">
+      <c r="C11" s="67">
         <v>2080</v>
       </c>
-      <c r="D11" s="71"/>
-      <c r="E11" s="70">
+      <c r="D11" s="68"/>
+      <c r="E11" s="67">
         <v>2150</v>
       </c>
-      <c r="F11" s="71"/>
-      <c r="G11" s="75">
+      <c r="F11" s="68"/>
+      <c r="G11" s="33">
         <v>2390</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <v>6</v>
       </c>
-      <c r="C12" s="70">
+      <c r="C12" s="67">
         <v>2320</v>
       </c>
-      <c r="D12" s="71"/>
-      <c r="E12" s="70">
+      <c r="D12" s="68"/>
+      <c r="E12" s="67">
         <v>2370</v>
       </c>
-      <c r="F12" s="71"/>
-      <c r="G12" s="75">
+      <c r="F12" s="68"/>
+      <c r="G12" s="33">
         <v>2620</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B13" s="5">
+      <c r="B13" s="4">
         <v>7</v>
       </c>
-      <c r="C13" s="70">
+      <c r="C13" s="67">
         <v>2560</v>
       </c>
-      <c r="D13" s="71"/>
-      <c r="E13" s="70">
+      <c r="D13" s="68"/>
+      <c r="E13" s="67">
         <v>2550</v>
       </c>
-      <c r="F13" s="71"/>
-      <c r="G13" s="75">
+      <c r="F13" s="68"/>
+      <c r="G13" s="33">
         <v>2880</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="7">
+      <c r="B14" s="6">
         <v>8</v>
       </c>
-      <c r="C14" s="68">
+      <c r="C14" s="71">
         <v>2800</v>
       </c>
-      <c r="D14" s="69"/>
-      <c r="E14" s="68">
+      <c r="D14" s="72"/>
+      <c r="E14" s="71">
         <v>2850</v>
       </c>
-      <c r="F14" s="69"/>
-      <c r="G14" s="76">
+      <c r="F14" s="72"/>
+      <c r="G14" s="34">
         <v>3100</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
     </row>
     <row r="17" spans="2:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="2:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="36" t="s">
+      <c r="B18" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="77"/>
-      <c r="D18" s="77"/>
-      <c r="E18" s="77"/>
-      <c r="F18" s="77"/>
-      <c r="G18" s="78"/>
+      <c r="C18" s="61"/>
+      <c r="D18" s="61"/>
+      <c r="E18" s="61"/>
+      <c r="F18" s="61"/>
+      <c r="G18" s="62"/>
     </row>
     <row r="19" spans="2:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="G19" s="18" t="s">
+      <c r="G19" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="I19" s="3" t="s">
+      <c r="I19" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B20" s="13">
+      <c r="B20" s="8">
         <v>1</v>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="13">
         <v>1170</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="13">
         <v>1150</v>
       </c>
-      <c r="E20" s="24">
+      <c r="E20" s="15">
         <v>1350</v>
       </c>
-      <c r="F20" s="21">
+      <c r="F20" s="73">
         <v>1040</v>
       </c>
-      <c r="G20" s="79"/>
+      <c r="G20" s="74"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B21" s="5">
+      <c r="B21" s="4">
         <v>2</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="1">
         <v>1350</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>1310</v>
       </c>
-      <c r="E21" s="25">
+      <c r="E21" s="16">
         <v>1580</v>
       </c>
-      <c r="F21" s="20">
+      <c r="F21" s="65">
         <v>1264</v>
       </c>
-      <c r="G21" s="42"/>
+      <c r="G21" s="66"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B22" s="5">
+      <c r="B22" s="4">
         <v>3</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="1">
         <v>1530</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>1460</v>
       </c>
-      <c r="E22" s="25">
+      <c r="E22" s="16">
         <v>1800</v>
       </c>
-      <c r="F22" s="20">
+      <c r="F22" s="65">
         <v>1489</v>
       </c>
-      <c r="G22" s="42"/>
+      <c r="G22" s="66"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B23" s="5">
+      <c r="B23" s="4">
         <v>4</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="1">
         <v>1700</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>1620</v>
       </c>
-      <c r="E23" s="25">
+      <c r="E23" s="16">
         <v>2030</v>
       </c>
-      <c r="F23" s="20">
+      <c r="F23" s="65">
         <v>1713</v>
       </c>
-      <c r="G23" s="42"/>
+      <c r="G23" s="66"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B24" s="5">
+      <c r="B24" s="4">
         <v>5</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="1">
         <v>1890</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="1">
         <v>1770</v>
       </c>
-      <c r="E24" s="25">
+      <c r="E24" s="16">
         <v>2250</v>
       </c>
-      <c r="F24" s="20">
+      <c r="F24" s="65">
         <v>1937</v>
       </c>
-      <c r="G24" s="42"/>
+      <c r="G24" s="66"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B25" s="5">
+      <c r="B25" s="4">
         <v>6</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C25" s="1">
         <v>2060</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="1">
         <v>1930</v>
       </c>
-      <c r="E25" s="25">
+      <c r="E25" s="16">
         <v>2480</v>
       </c>
-      <c r="F25" s="20">
+      <c r="F25" s="65">
         <v>2161</v>
       </c>
-      <c r="G25" s="42"/>
+      <c r="G25" s="66"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="B26" s="5">
+      <c r="B26" s="4">
         <v>7</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C26" s="1">
         <v>2240</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>2080</v>
       </c>
-      <c r="E26" s="25">
+      <c r="E26" s="16">
         <v>2700</v>
       </c>
-      <c r="F26" s="20">
+      <c r="F26" s="65">
         <v>2386</v>
       </c>
-      <c r="G26" s="42"/>
+      <c r="G26" s="66"/>
     </row>
     <row r="27" spans="2:9" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="7">
+      <c r="B27" s="6">
         <v>8</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="14">
         <v>2420</v>
       </c>
-      <c r="D27" s="23">
+      <c r="D27" s="14">
         <v>2240</v>
       </c>
-      <c r="E27" s="26">
+      <c r="E27" s="17">
         <v>2930</v>
       </c>
-      <c r="F27" s="43">
+      <c r="F27" s="63">
         <v>2610</v>
       </c>
-      <c r="G27" s="44"/>
+      <c r="G27" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="B5:G5"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="E7:F7"/>
@@ -2333,15 +2357,19 @@
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F24:G24"/>
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="F22:G22"/>
     <mergeCell ref="F21:G21"/>
-    <mergeCell ref="E13:F13"/>
     <mergeCell ref="F20:G20"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="B5:G5"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2359,340 +2387,332 @@
   <sheetData>
     <row r="4" spans="2:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="12"/>
+      <c r="C5" s="76"/>
+      <c r="D5" s="76"/>
+      <c r="E5" s="76"/>
+      <c r="F5" s="76"/>
+      <c r="G5" s="76"/>
+      <c r="H5" s="77"/>
     </row>
     <row r="6" spans="2:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="G6" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B7" s="13">
+      <c r="B7" s="8">
         <v>1</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="85">
         <v>1107</v>
       </c>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14">
+      <c r="D7" s="85"/>
+      <c r="E7" s="85"/>
+      <c r="F7" s="85">
         <v>1457</v>
       </c>
-      <c r="G7" s="14"/>
-      <c r="H7" s="15">
+      <c r="G7" s="85"/>
+      <c r="H7" s="9">
         <v>1473</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="83">
         <v>1422</v>
       </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1">
+      <c r="D8" s="83"/>
+      <c r="E8" s="83"/>
+      <c r="F8" s="83">
         <v>1610</v>
       </c>
-      <c r="G8" s="1"/>
-      <c r="H8" s="6">
+      <c r="G8" s="83"/>
+      <c r="H8" s="5">
         <v>1660</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B9" s="5">
+      <c r="B9" s="4">
         <v>3</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="83">
         <v>1675</v>
       </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1">
+      <c r="D9" s="83"/>
+      <c r="E9" s="83"/>
+      <c r="F9" s="83">
         <v>1740</v>
       </c>
-      <c r="G9" s="1"/>
-      <c r="H9" s="6">
+      <c r="G9" s="83"/>
+      <c r="H9" s="5">
         <v>1940</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B10" s="5">
+      <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="83">
         <v>1921</v>
       </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1">
+      <c r="D10" s="83"/>
+      <c r="E10" s="83"/>
+      <c r="F10" s="83">
         <v>1960</v>
       </c>
-      <c r="G10" s="1"/>
-      <c r="H10" s="6">
+      <c r="G10" s="83"/>
+      <c r="H10" s="5">
         <v>2120</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>5</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="83">
         <v>2170</v>
       </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1">
+      <c r="D11" s="83"/>
+      <c r="E11" s="83"/>
+      <c r="F11" s="83">
         <v>2150</v>
       </c>
-      <c r="G11" s="1"/>
-      <c r="H11" s="6">
+      <c r="G11" s="83"/>
+      <c r="H11" s="5">
         <v>2390</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <v>6</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12" s="83">
         <v>2440</v>
       </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1">
+      <c r="D12" s="83"/>
+      <c r="E12" s="83"/>
+      <c r="F12" s="83">
         <v>2370</v>
       </c>
-      <c r="G12" s="1"/>
-      <c r="H12" s="6">
+      <c r="G12" s="83"/>
+      <c r="H12" s="5">
         <v>2620</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.3">
-      <c r="B13" s="5">
+      <c r="B13" s="4">
         <v>7</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="83">
         <v>2710</v>
       </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1">
+      <c r="D13" s="83"/>
+      <c r="E13" s="83"/>
+      <c r="F13" s="83">
         <v>2550</v>
       </c>
-      <c r="G13" s="1"/>
-      <c r="H13" s="6">
+      <c r="G13" s="83"/>
+      <c r="H13" s="5">
         <v>2880</v>
       </c>
     </row>
     <row r="14" spans="2:10" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="7">
+      <c r="B14" s="6">
         <v>8</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="81">
         <v>3000</v>
       </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8">
+      <c r="D14" s="81"/>
+      <c r="E14" s="81"/>
+      <c r="F14" s="81">
         <v>2850</v>
       </c>
-      <c r="G14" s="8"/>
-      <c r="H14" s="9">
+      <c r="G14" s="81"/>
+      <c r="H14" s="7">
         <v>3100</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="30"/>
+      <c r="C18" s="79"/>
+      <c r="D18" s="79"/>
+      <c r="E18" s="79"/>
+      <c r="F18" s="80"/>
     </row>
     <row r="19" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="G19" s="49"/>
-      <c r="H19" s="34" t="s">
+      <c r="G19" s="25"/>
+      <c r="H19" s="20" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B20" s="13">
+      <c r="B20" s="8">
         <v>1</v>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="13">
         <v>1210</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="13">
         <v>1170</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="85">
         <v>1040</v>
       </c>
-      <c r="F20" s="31"/>
+      <c r="F20" s="86"/>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B21" s="5">
+      <c r="B21" s="4">
         <v>2</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="1">
         <v>1420</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>1370</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="83">
         <v>1264</v>
       </c>
-      <c r="F21" s="32"/>
+      <c r="F21" s="84"/>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B22" s="5">
+      <c r="B22" s="4">
         <v>3</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22" s="1">
         <v>1630</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>1570</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22" s="83">
         <v>1489</v>
       </c>
-      <c r="F22" s="32"/>
+      <c r="F22" s="84"/>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B23" s="5">
+      <c r="B23" s="4">
         <v>4</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23" s="1">
         <v>1840</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>1770</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="83">
         <v>1713</v>
       </c>
-      <c r="F23" s="32"/>
+      <c r="F23" s="84"/>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B24" s="5">
+      <c r="B24" s="4">
         <v>5</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C24" s="1">
         <v>2050</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="1">
         <v>1970</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24" s="83">
         <v>1937</v>
       </c>
-      <c r="F24" s="32"/>
+      <c r="F24" s="84"/>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B25" s="5">
+      <c r="B25" s="4">
         <v>6</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C25" s="1">
         <v>2260</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="1">
         <v>2170</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25" s="83">
         <v>2161</v>
       </c>
-      <c r="F25" s="32"/>
+      <c r="F25" s="84"/>
     </row>
     <row r="26" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B26" s="5">
+      <c r="B26" s="4">
         <v>7</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C26" s="1">
         <v>2470</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="1">
         <v>2370</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="83">
         <v>2386</v>
       </c>
-      <c r="F26" s="32"/>
+      <c r="F26" s="84"/>
     </row>
     <row r="27" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="7">
+      <c r="B27" s="6">
         <v>8</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="14">
         <v>2700</v>
       </c>
-      <c r="D27" s="23">
+      <c r="D27" s="14">
         <v>2600</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27" s="81">
         <v>2610</v>
       </c>
-      <c r="F27" s="33"/>
+      <c r="F27" s="82"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="E27:F27"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="C9:E9"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="C7:E7"/>
@@ -2709,7 +2729,15 @@
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="C11:E11"/>
     <mergeCell ref="C10:E10"/>
-    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="E27:F27"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E20:F20"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2727,78 +2755,78 @@
   <sheetData>
     <row r="4" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="75" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="12"/>
+      <c r="C5" s="101"/>
+      <c r="D5" s="101"/>
+      <c r="E5" s="76"/>
+      <c r="F5" s="76"/>
+      <c r="G5" s="76"/>
+      <c r="H5" s="77"/>
     </row>
     <row r="6" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="37" t="s">
+      <c r="B6" s="91" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="45" t="s">
+      <c r="G6" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="48"/>
-      <c r="J6" s="3" t="s">
+      <c r="H6" s="88"/>
+      <c r="J6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="L6" s="34" t="s">
+      <c r="L6" s="20" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="38"/>
-      <c r="C7" s="45" t="s">
+      <c r="B7" s="92"/>
+      <c r="C7" s="87" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="46"/>
-      <c r="E7" s="47" t="s">
+      <c r="D7" s="93"/>
+      <c r="E7" s="94" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="48"/>
-      <c r="G7" s="16" t="s">
+      <c r="F7" s="88"/>
+      <c r="G7" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="18" t="s">
+      <c r="H7" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="J7" s="34"/>
-      <c r="L7" s="34"/>
+      <c r="J7" s="20"/>
+      <c r="L7" s="20"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B8" s="39">
+      <c r="B8" s="22">
         <v>1</v>
       </c>
-      <c r="C8" s="50">
+      <c r="C8" s="102">
         <v>4</v>
       </c>
-      <c r="D8" s="51"/>
-      <c r="E8" s="56">
+      <c r="D8" s="103"/>
+      <c r="E8" s="104">
         <v>18</v>
       </c>
-      <c r="F8" s="57"/>
-      <c r="G8" s="65">
+      <c r="F8" s="105"/>
+      <c r="G8" s="29">
         <v>4</v>
       </c>
-      <c r="H8" s="62">
+      <c r="H8" s="26">
         <v>18</v>
       </c>
       <c r="L8" t="s">
@@ -2806,161 +2834,161 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="40">
+      <c r="B9" s="23">
         <v>2</v>
       </c>
-      <c r="C9" s="52">
+      <c r="C9" s="97">
         <v>5.2</v>
       </c>
-      <c r="D9" s="53"/>
-      <c r="E9" s="58">
+      <c r="D9" s="98"/>
+      <c r="E9" s="89">
         <v>28</v>
       </c>
-      <c r="F9" s="59"/>
-      <c r="G9" s="66">
+      <c r="F9" s="90"/>
+      <c r="G9" s="30">
         <v>5.2</v>
       </c>
-      <c r="H9" s="63">
+      <c r="H9" s="27">
         <v>28</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B10" s="40">
+      <c r="B10" s="23">
         <v>3</v>
       </c>
-      <c r="C10" s="52">
+      <c r="C10" s="97">
         <v>6.5</v>
       </c>
-      <c r="D10" s="53"/>
-      <c r="E10" s="58">
+      <c r="D10" s="98"/>
+      <c r="E10" s="89">
         <v>39</v>
       </c>
-      <c r="F10" s="59"/>
-      <c r="G10" s="66">
+      <c r="F10" s="90"/>
+      <c r="G10" s="30">
         <v>6.5</v>
       </c>
-      <c r="H10" s="63">
+      <c r="H10" s="27">
         <v>39</v>
       </c>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B11" s="40">
+      <c r="B11" s="23">
         <v>4</v>
       </c>
-      <c r="C11" s="52">
+      <c r="C11" s="97">
         <v>7.7</v>
       </c>
-      <c r="D11" s="53"/>
-      <c r="E11" s="58">
+      <c r="D11" s="98"/>
+      <c r="E11" s="89">
         <v>49</v>
       </c>
-      <c r="F11" s="59"/>
-      <c r="G11" s="66">
+      <c r="F11" s="90"/>
+      <c r="G11" s="30">
         <v>7.7</v>
       </c>
-      <c r="H11" s="63">
+      <c r="H11" s="27">
         <v>49</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B12" s="40">
+      <c r="B12" s="23">
         <v>5</v>
       </c>
-      <c r="C12" s="52">
+      <c r="C12" s="97">
         <v>9</v>
       </c>
-      <c r="D12" s="53"/>
-      <c r="E12" s="58">
+      <c r="D12" s="98"/>
+      <c r="E12" s="89">
         <v>60</v>
       </c>
-      <c r="F12" s="59"/>
-      <c r="G12" s="66">
+      <c r="F12" s="90"/>
+      <c r="G12" s="30">
         <v>9</v>
       </c>
-      <c r="H12" s="63">
+      <c r="H12" s="27">
         <v>60</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B13" s="40">
+      <c r="B13" s="23">
         <v>6</v>
       </c>
-      <c r="C13" s="52">
+      <c r="C13" s="97">
         <v>10.199999999999999</v>
       </c>
-      <c r="D13" s="53"/>
-      <c r="E13" s="58">
+      <c r="D13" s="98"/>
+      <c r="E13" s="89">
         <v>70</v>
       </c>
-      <c r="F13" s="59"/>
-      <c r="G13" s="66">
+      <c r="F13" s="90"/>
+      <c r="G13" s="30">
         <v>10.199999999999999</v>
       </c>
-      <c r="H13" s="63">
+      <c r="H13" s="27">
         <v>70</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B14" s="40">
+      <c r="B14" s="23">
         <v>7</v>
       </c>
-      <c r="C14" s="52">
+      <c r="C14" s="97">
         <v>11.3</v>
       </c>
-      <c r="D14" s="53"/>
-      <c r="E14" s="58">
+      <c r="D14" s="98"/>
+      <c r="E14" s="89">
         <v>79</v>
       </c>
-      <c r="F14" s="59"/>
-      <c r="G14" s="66">
+      <c r="F14" s="90"/>
+      <c r="G14" s="30">
         <v>10.8</v>
       </c>
-      <c r="H14" s="63">
+      <c r="H14" s="27">
         <v>75</v>
       </c>
     </row>
     <row r="15" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="41">
+      <c r="B15" s="24">
         <v>8</v>
       </c>
-      <c r="C15" s="54">
+      <c r="C15" s="95">
         <v>13.5</v>
       </c>
-      <c r="D15" s="55"/>
-      <c r="E15" s="60">
+      <c r="D15" s="96"/>
+      <c r="E15" s="99">
         <v>92</v>
       </c>
-      <c r="F15" s="61"/>
-      <c r="G15" s="67">
+      <c r="F15" s="100"/>
+      <c r="G15" s="31">
         <v>13.5</v>
       </c>
-      <c r="H15" s="64">
+      <c r="H15" s="28">
         <v>92</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C11:D11"/>
     <mergeCell ref="E15:F15"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:F8"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E12:F12"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2979,146 +3007,149 @@
   <sheetData>
     <row r="4" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="75" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="12"/>
+      <c r="C5" s="101"/>
+      <c r="D5" s="101"/>
+      <c r="E5" s="76"/>
+      <c r="F5" s="76"/>
+      <c r="G5" s="76"/>
+      <c r="H5" s="77"/>
     </row>
     <row r="6" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="80" t="s">
+      <c r="B6" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="81" t="s">
+      <c r="C6" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="45" t="s">
+      <c r="G6" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="48"/>
-      <c r="L6" s="34"/>
+      <c r="H6" s="88"/>
+      <c r="L6" s="20"/>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B7" s="39">
+      <c r="B7" s="22">
         <v>1</v>
       </c>
-      <c r="C7" s="108">
+      <c r="C7" s="113">
         <v>1200</v>
       </c>
-      <c r="D7" s="109"/>
-      <c r="E7" s="21">
+      <c r="D7" s="114"/>
+      <c r="E7" s="73">
         <v>1390</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="79"/>
+      <c r="F7" s="109"/>
+      <c r="G7" s="109"/>
+      <c r="H7" s="74"/>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B8" s="40">
+      <c r="B8" s="23">
         <v>2</v>
       </c>
       <c r="C8" s="110">
         <v>1570</v>
       </c>
-      <c r="D8" s="112"/>
-      <c r="E8" s="112"/>
-      <c r="F8" s="112"/>
-      <c r="G8" s="112"/>
-      <c r="H8" s="113"/>
+      <c r="D8" s="111"/>
+      <c r="E8" s="111"/>
+      <c r="F8" s="111"/>
+      <c r="G8" s="111"/>
+      <c r="H8" s="112"/>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="40">
+      <c r="B9" s="23">
         <v>3</v>
       </c>
       <c r="C9" s="110">
         <v>1840</v>
       </c>
-      <c r="D9" s="112"/>
-      <c r="E9" s="112"/>
-      <c r="F9" s="112"/>
-      <c r="G9" s="112"/>
-      <c r="H9" s="113"/>
+      <c r="D9" s="111"/>
+      <c r="E9" s="111"/>
+      <c r="F9" s="111"/>
+      <c r="G9" s="111"/>
+      <c r="H9" s="112"/>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B10" s="40">
+      <c r="B10" s="23">
         <v>4</v>
       </c>
       <c r="C10" s="110">
         <v>2110</v>
       </c>
-      <c r="D10" s="112"/>
-      <c r="E10" s="112"/>
-      <c r="F10" s="112"/>
-      <c r="G10" s="112"/>
-      <c r="H10" s="113"/>
+      <c r="D10" s="111"/>
+      <c r="E10" s="111"/>
+      <c r="F10" s="111"/>
+      <c r="G10" s="111"/>
+      <c r="H10" s="112"/>
     </row>
     <row r="11" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B11" s="40">
+      <c r="B11" s="23">
         <v>5</v>
       </c>
       <c r="C11" s="110">
         <v>2380</v>
       </c>
-      <c r="D11" s="112"/>
-      <c r="E11" s="112"/>
-      <c r="F11" s="112"/>
-      <c r="G11" s="112"/>
-      <c r="H11" s="113"/>
+      <c r="D11" s="111"/>
+      <c r="E11" s="111"/>
+      <c r="F11" s="111"/>
+      <c r="G11" s="111"/>
+      <c r="H11" s="112"/>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B12" s="40">
+      <c r="B12" s="23">
         <v>6</v>
       </c>
       <c r="C12" s="110">
         <v>2650</v>
       </c>
-      <c r="D12" s="112"/>
-      <c r="E12" s="112"/>
-      <c r="F12" s="112"/>
-      <c r="G12" s="112"/>
-      <c r="H12" s="113"/>
+      <c r="D12" s="111"/>
+      <c r="E12" s="111"/>
+      <c r="F12" s="111"/>
+      <c r="G12" s="111"/>
+      <c r="H12" s="112"/>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B13" s="40">
+      <c r="B13" s="23">
         <v>7</v>
       </c>
       <c r="C13" s="110">
         <v>2920</v>
       </c>
-      <c r="D13" s="112"/>
-      <c r="E13" s="112"/>
-      <c r="F13" s="112"/>
-      <c r="G13" s="112"/>
-      <c r="H13" s="113"/>
+      <c r="D13" s="111"/>
+      <c r="E13" s="111"/>
+      <c r="F13" s="111"/>
+      <c r="G13" s="111"/>
+      <c r="H13" s="112"/>
     </row>
     <row r="14" spans="2:12" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="41">
+      <c r="B14" s="24">
         <v>8</v>
       </c>
-      <c r="C14" s="111">
+      <c r="C14" s="106">
         <v>3190</v>
       </c>
-      <c r="D14" s="114"/>
-      <c r="E14" s="114"/>
-      <c r="F14" s="114"/>
-      <c r="G14" s="114"/>
-      <c r="H14" s="115"/>
+      <c r="D14" s="107"/>
+      <c r="E14" s="107"/>
+      <c r="F14" s="107"/>
+      <c r="G14" s="107"/>
+      <c r="H14" s="108"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="C7:D7"/>
     <mergeCell ref="C14:H14"/>
     <mergeCell ref="E7:H7"/>
     <mergeCell ref="C11:H11"/>
@@ -3127,9 +3158,6 @@
     <mergeCell ref="C8:H8"/>
     <mergeCell ref="C9:H9"/>
     <mergeCell ref="C10:H10"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="C7:D7"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3147,28 +3175,28 @@
   <sheetData>
     <row r="4" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="82" t="s">
+      <c r="B5" s="115" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="83"/>
-      <c r="F5" s="3" t="s">
+      <c r="C5" s="116"/>
+      <c r="F5" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="34"/>
+      <c r="G6" s="20"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B7" s="13">
+      <c r="B7" s="8">
         <v>1</v>
       </c>
-      <c r="C7" s="84">
+      <c r="C7" s="37">
         <v>1200</v>
       </c>
       <c r="D7" t="s">
@@ -3176,58 +3204,58 @@
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="85">
+      <c r="C8" s="38">
         <v>1454</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B9" s="5">
+      <c r="B9" s="4">
         <v>3</v>
       </c>
-      <c r="C9" s="85">
+      <c r="C9" s="38">
         <v>1708</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B10" s="5">
+      <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="85">
+      <c r="C10" s="38">
         <v>1962</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>5</v>
       </c>
-      <c r="C11" s="85">
+      <c r="C11" s="38">
         <v>2216</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <v>6</v>
       </c>
-      <c r="C12" s="85">
+      <c r="C12" s="38">
         <v>2470</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B13" s="5">
+      <c r="B13" s="4">
         <v>7</v>
       </c>
-      <c r="C13" s="85">
+      <c r="C13" s="38">
         <v>2724</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="7">
+      <c r="B14" s="6">
         <v>8</v>
       </c>
-      <c r="C14" s="86">
+      <c r="C14" s="39">
         <v>2980</v>
       </c>
       <c r="D14" t="s">
@@ -3254,81 +3282,81 @@
   <sheetData>
     <row r="4" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="82" t="s">
+      <c r="B5" s="115" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="83"/>
+      <c r="C5" s="116"/>
     </row>
     <row r="6" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="34"/>
+      <c r="G6" s="20"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B7" s="13">
+      <c r="B7" s="8">
         <v>1</v>
       </c>
-      <c r="C7" s="84">
+      <c r="C7" s="37">
         <v>1200</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="85">
+      <c r="C8" s="38">
         <v>1454</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B9" s="5">
+      <c r="B9" s="4">
         <v>3</v>
       </c>
-      <c r="C9" s="85">
+      <c r="C9" s="38">
         <v>1708</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B10" s="5">
+      <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="85">
+      <c r="C10" s="38">
         <v>1962</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>5</v>
       </c>
-      <c r="C11" s="85">
+      <c r="C11" s="38">
         <v>2216</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <v>6</v>
       </c>
-      <c r="C12" s="85">
+      <c r="C12" s="38">
         <v>2470</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B13" s="5">
+      <c r="B13" s="4">
         <v>7</v>
       </c>
-      <c r="C13" s="85">
+      <c r="C13" s="38">
         <v>2724</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="7">
+      <c r="B14" s="6">
         <v>8</v>
       </c>
-      <c r="C14" s="86">
+      <c r="C14" s="39">
         <v>2980</v>
       </c>
     </row>
@@ -3352,84 +3380,84 @@
   <sheetData>
     <row r="4" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="82" t="s">
+      <c r="B5" s="115" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="107"/>
+      <c r="C5" s="117"/>
     </row>
     <row r="6" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="E6" s="34" t="s">
+      <c r="E6" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="G6" s="34"/>
+      <c r="G6" s="20"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B7" s="13">
+      <c r="B7" s="8">
         <v>1</v>
       </c>
-      <c r="C7" s="84">
+      <c r="C7" s="37">
         <v>1100</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <v>2</v>
       </c>
-      <c r="C8" s="85">
+      <c r="C8" s="38">
         <v>1340</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B9" s="5">
+      <c r="B9" s="4">
         <v>3</v>
       </c>
-      <c r="C9" s="85">
+      <c r="C9" s="38">
         <v>1600</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B10" s="5">
+      <c r="B10" s="4">
         <v>4</v>
       </c>
-      <c r="C10" s="85">
+      <c r="C10" s="38">
         <v>1810</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B11" s="5">
+      <c r="B11" s="4">
         <v>5</v>
       </c>
-      <c r="C11" s="85">
+      <c r="C11" s="38">
         <v>2050</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B12" s="5">
+      <c r="B12" s="4">
         <v>6</v>
       </c>
-      <c r="C12" s="85">
+      <c r="C12" s="38">
         <v>2320</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
-      <c r="B13" s="5">
+      <c r="B13" s="4">
         <v>7</v>
       </c>
-      <c r="C13" s="85">
+      <c r="C13" s="38">
         <v>2610</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="7">
+      <c r="B14" s="6">
         <v>8</v>
       </c>
-      <c r="C14" s="86">
+      <c r="C14" s="39">
         <v>2930</v>
       </c>
     </row>
@@ -3441,4 +3469,137 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B4:H14"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="4" width="11.625" customWidth="1"/>
+    <col min="6" max="6" width="41.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="115" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="118"/>
+      <c r="D5" s="116"/>
+    </row>
+    <row r="6" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="119" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="20"/>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B7" s="8">
+        <v>1</v>
+      </c>
+      <c r="C7" s="37">
+        <v>970</v>
+      </c>
+      <c r="D7" s="37">
+        <v>1210</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B8" s="4">
+        <v>2</v>
+      </c>
+      <c r="C8" s="38">
+        <v>1220</v>
+      </c>
+      <c r="D8" s="38">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B9" s="4">
+        <v>3</v>
+      </c>
+      <c r="C9" s="38">
+        <v>1460</v>
+      </c>
+      <c r="D9" s="38">
+        <v>1760</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B10" s="4">
+        <v>4</v>
+      </c>
+      <c r="C10" s="38">
+        <v>1690</v>
+      </c>
+      <c r="D10" s="38">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B11" s="4">
+        <v>5</v>
+      </c>
+      <c r="C11" s="38">
+        <v>1985</v>
+      </c>
+      <c r="D11" s="38">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B12" s="4">
+        <v>6</v>
+      </c>
+      <c r="C12" s="38">
+        <v>2280</v>
+      </c>
+      <c r="D12" s="38">
+        <v>2610</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B13" s="4">
+        <v>7</v>
+      </c>
+      <c r="C13" s="38">
+        <v>2860</v>
+      </c>
+      <c r="D13" s="38">
+        <v>2920</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="6">
+        <v>8</v>
+      </c>
+      <c r="C14" s="39">
+        <v>3250</v>
+      </c>
+      <c r="D14" s="39">
+        <v>3110</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B5:D5"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>